<commit_message>
feat: implementar requisito 6.1 para qualidade e ambiente
</commit_message>
<xml_diff>
--- a/public/documents/requirement6/6_1/6_1_modelo_aspetos_ambiental.xlsx
+++ b/public/documents/requirement6/6_1/6_1_modelo_aspetos_ambiental.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiff\Tec. Qualidade e Sustentabilidade\Sistema de Gestão Ambiental (SGA)\6. Planeamento\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiff\integra-sgi\integra-sgi\public\documents\requirement6\6_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BB280D2-C4C0-40C8-A90F-8BEA115E47E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC23799-1493-4F87-9A81-DD687749FBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{073A7DA1-8F09-4975-A959-95672E64B932}"/>
   </bookViews>
   <sheets>
-    <sheet name="Folha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Aspetos Ambientais" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="53">
-  <si>
-    <t>AVALIAÇÃO DA SIGNIFICÂNCIA DOS ASPETOS AMBIENTAIS</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Aspeto Ambiental (Causa)</t>
   </si>
@@ -59,142 +56,13 @@
     <t>Significância</t>
   </si>
   <si>
-    <t>Deposição em aterro / Esgotamento de solos</t>
-  </si>
-  <si>
-    <t>Significativo</t>
-  </si>
-  <si>
-    <t>Esgotamento de recursos hídricos</t>
-  </si>
-  <si>
-    <t>Moderado</t>
-  </si>
-  <si>
-    <t>Poluição de linhas de água (DGO/DQO)</t>
-  </si>
-  <si>
-    <t>Destruição da camada de ozono / Aquecimento global</t>
-  </si>
-  <si>
-    <t>Poluição sonora (vizinhança de Coimbra)</t>
-  </si>
-  <si>
-    <t>Acumulação de resíduos não biodegradáveis</t>
-  </si>
-  <si>
-    <t>Contaminação química do solo/água</t>
-  </si>
-  <si>
-    <t>Baixo</t>
-  </si>
-  <si>
-    <t>Poluição atmosférica local</t>
-  </si>
-  <si>
-    <t>Contaminação por metais pesados</t>
-  </si>
-  <si>
-    <t>Emissões indiretas de CO2</t>
-  </si>
-  <si>
     <t>Critério de Gravidade</t>
   </si>
   <si>
     <t>Critério de Probabilidade</t>
   </si>
   <si>
-    <t>(Constante): Gerados em todos os turnos de desmancha.</t>
-  </si>
-  <si>
-    <t>(Constante): Uso obrigatório para higiene e refrigeração diária.</t>
-  </si>
-  <si>
-    <t>(Frequente): Lavagem diária das linhas de abate/desmancha.</t>
-  </si>
-  <si>
-    <t>(Improvável): Ocorre apenas em caso de fuga ou manutenção.</t>
-  </si>
-  <si>
-    <t>(Constante): As câmaras de frio nunca desligam (24/7).</t>
-  </si>
-  <si>
-    <t>(Frequente): Funcionamento contínuo das máquinas de frio.</t>
-  </si>
-  <si>
-    <t>(Constante): Todo o produto final é embalado para venda.</t>
-  </si>
-  <si>
-    <t>(Improvável): Manuseamento de detergentes concentrados é controlado.</t>
-  </si>
-  <si>
-    <t>(Frequente): Expedição diária de mercadorias em camiões térmicos.</t>
-  </si>
-  <si>
-    <t>(Improvável): Gerados apenas em manutenção pontual.</t>
-  </si>
-  <si>
-    <t>(Moderado): Impacto significativo no volume de resíduos, mas com destino autorizado.</t>
-  </si>
-  <si>
-    <t>(Menor): Recurso escasso, mas o impacto individual por litro é baixo.</t>
-  </si>
-  <si>
-    <t>(Grave): Elevada carga poluidora (DQO/DBO); risco de multas da APA/ASAE.</t>
-  </si>
-  <si>
-    <t>(Grave): Alto Potencial de Aquecimento Global (GWP) e custo de reposição.</t>
-  </si>
-  <si>
-    <t>(Moderado): Elevada pegada de carbono e custo operacional fixo.</t>
-  </si>
-  <si>
-    <t>(Menor): Impacto limitado à vizinhança imediata em Coimbra.</t>
-  </si>
-  <si>
-    <t>(Menor): Impacto disperso, mas os materiais são recicláveis (Ponto Verde).</t>
-  </si>
-  <si>
-    <t>(Moderado): Pode contaminar a ETAR se for em grande volume.</t>
-  </si>
-  <si>
-    <t>(Moderado): Emissão local de NOₓ e CO₂ em zonas urbanas.</t>
-  </si>
-  <si>
-    <t>(Moderado): Perigosos se misturados com o lixo comum (metais pesados).</t>
-  </si>
-  <si>
     <t>ID</t>
-  </si>
-  <si>
-    <t>Produção de subprodutos (ossos, gorduras)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Consumo de água (lavagem de carcaças e pavimentos)</t>
-  </si>
-  <si>
-    <t>Rejeição de efluentes com sangue/matéria orgânica</t>
-  </si>
-  <si>
-    <t>Emissões de gases refrigerantes (fugas de F-Gases)</t>
-  </si>
-  <si>
-    <t>Consumo de energia elétrica (câmaras de frio 24h)</t>
-  </si>
-  <si>
-    <t>Ruído das unidades condensadoras e logística</t>
-  </si>
-  <si>
-    <t>Produção de embalagens plásticas e filmes</t>
-  </si>
-  <si>
-    <t>Derrame acidental de produtos de limpeza (detergentes)</t>
-  </si>
-  <si>
-    <t>Emissões de veículos de transporte (gasóleo)</t>
-  </si>
-  <si>
-    <t>Descarte de lâmpadas ou resíduos eletrónicos (E-Waste)</t>
   </si>
 </sst>
 </file>
@@ -245,13 +113,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF814E1D"/>
+        <fgColor rgb="FF203E5E"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFAA0106"/>
+        <fgColor rgb="FF0F7343"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -356,6 +224,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -364,9 +235,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -437,6 +305,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF0F7343"/>
+      <color rgb="FF203E5E"/>
       <color rgb="FFAA0106"/>
       <color rgb="FF814E1D"/>
       <color rgb="FF420D07"/>
@@ -457,23 +327,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>53786</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>537883</xdr:colOff>
+      <xdr:colOff>80682</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>170180</xdr:rowOff>
+      <xdr:rowOff>98613</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagem 3">
+        <xdr:cNvPr id="3" name="Imagem 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FEF5501-FA1F-53D1-E187-9FAFA36A508D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{53ECC2C1-ADEB-39A7-A840-438664F71306}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -495,8 +365,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1844040" cy="1229360"/>
+          <a:off x="125504" y="0"/>
+          <a:ext cx="1192307" cy="1192307"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -830,7 +700,7 @@
   <cols>
     <col min="1" max="1" width="1" style="1" customWidth="1"/>
     <col min="2" max="2" width="17" style="1" customWidth="1"/>
-    <col min="3" max="3" width="24.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26.21875" style="1" customWidth="1"/>
     <col min="4" max="4" width="37.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.77734375" style="1" customWidth="1"/>
     <col min="6" max="6" width="32.109375" style="1" bestFit="1" customWidth="1"/>
@@ -841,336 +711,154 @@
     <col min="11" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="11" t="s">
+    <row r="2" spans="2:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+    </row>
+    <row r="4" spans="2:10" ht="30" x14ac:dyDescent="0.3">
+      <c r="B4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-    </row>
-    <row r="4" spans="2:10" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>21</v>
+      <c r="H4" s="11" t="s">
+        <v>6</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="I4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="2">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="4">
-        <v>5</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="7">
-        <v>3</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" s="5">
-        <v>15</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2">
-        <v>2</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="4">
-        <v>5</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="7">
-        <v>2</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="5">
-        <v>10</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="2">
-        <v>3</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="4">
-        <v>4</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="7">
-        <v>4</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" s="5">
-        <v>16</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2">
-        <v>4</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="4">
-        <v>2</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="7">
-        <v>4</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I8" s="5">
-        <v>8</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B9" s="2">
-        <v>5</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="4">
-        <v>5</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G9" s="7">
-        <v>3</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="I9" s="5">
-        <v>15</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="2">
-        <v>6</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="4">
-        <v>4</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="7">
-        <v>2</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I10" s="5">
-        <v>8</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="2">
-        <v>7</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="4">
-        <v>5</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" s="7">
-        <v>2</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I11" s="5">
-        <v>10</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B12" s="2">
-        <v>8</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="4">
-        <v>2</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="7">
-        <v>3</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="I12" s="5">
-        <v>6</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="2">
-        <v>9</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="4">
-        <v>4</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="7">
-        <v>3</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="I13" s="5">
-        <v>12</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="2">
-        <v>10</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="4">
-        <v>2</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="7">
-        <v>3</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="I14" s="5">
-        <v>6</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>16</v>
-      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B6" s="2"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B7" s="2"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B8" s="2"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B9" s="2"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B10" s="2"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B11" s="2"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B12" s="2"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="3"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B13" s="2"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B14" s="2"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>